<commit_message>
PH SSB inputs and before producing PH effects costing scenarios
</commit_message>
<xml_diff>
--- a/data/indonesia_model_inputs.xlsx
+++ b/data/indonesia_model_inputs.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/WorldBank-Indonesia/uw-wb-indonesia-ncd/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_0C710D44475D1BAD4A588195A28C8E47DB0B7F50" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4580B05-CC0E-43C9-9064-322DEC044C63}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_0C710D44475D1BAD4A588195A28C8E47DB0B7F50" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8523B379-E550-4158-B9D4-5582EA6E3F24}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="Assumptions" sheetId="2" r:id="rId2"/>
-    <sheet name="Dictionaries" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="Intervention_Cause_Map" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="Dictionaries" sheetId="3" r:id="rId3"/>
+    <sheet name="Intervention_Cause_Map" sheetId="4" r:id="rId4"/>
     <sheet name="Effect_Sizes" sheetId="5" r:id="rId5"/>
     <sheet name="Coverage" sheetId="6" r:id="rId6"/>
     <sheet name="Cost_Components" sheetId="7" r:id="rId7"/>
     <sheet name="Model_Input_View" sheetId="8" r:id="rId8"/>
-    <sheet name="FairChoices_Methods" sheetId="9" state="hidden" r:id="rId9"/>
-    <sheet name="Scope_and_Sources" sheetId="10" state="hidden" r:id="rId10"/>
-    <sheet name="QA_Checks" sheetId="11" state="hidden" r:id="rId11"/>
+    <sheet name="FairChoices_Methods" sheetId="9" r:id="rId9"/>
+    <sheet name="Scope_and_Sources" sheetId="10" r:id="rId10"/>
+    <sheet name="QA_Checks" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2279,20 +2279,26 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2315,26 +2321,20 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3192,38 +3192,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="67"/>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
+      <c r="A2" s="55"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="68" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
+      <c r="A3" s="56" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1"/>
@@ -3236,54 +3236,54 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="69"/>
-      <c r="C5" s="69" t="s">
+      <c r="B5" s="57"/>
+      <c r="C5" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="69"/>
-      <c r="E5" s="69" t="s">
+      <c r="D5" s="57"/>
+      <c r="E5" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69" t="s">
+      <c r="F5" s="57"/>
+      <c r="G5" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="69"/>
+      <c r="H5" s="57"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="70" t="str">
+      <c r="A6" s="58" t="str">
         <f>IF(COUNTIF(QA_Checks!$E$2:$E$9,"FAIL")=0,"READY TO RUN","REVIEW REQUIRED")</f>
         <v>REVIEW REQUIRED</v>
       </c>
-      <c r="B6" s="71"/>
-      <c r="C6" s="70">
+      <c r="B6" s="59"/>
+      <c r="C6" s="58">
         <f>COUNTA(Dictionaries!$A$2:$A$9)</f>
         <v>8</v>
       </c>
-      <c r="D6" s="71"/>
-      <c r="E6" s="70">
+      <c r="D6" s="59"/>
+      <c r="E6" s="58">
         <f>COUNTIF(Dictionaries!$I$2:$I$9,1)</f>
         <v>7</v>
       </c>
-      <c r="F6" s="71"/>
-      <c r="G6" s="70">
+      <c r="F6" s="59"/>
+      <c r="G6" s="58">
         <f>COUNTA(Intervention_Cause_Map!$A$2:$A$18)</f>
         <v>17</v>
       </c>
-      <c r="H6" s="71"/>
+      <c r="H6" s="59"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="72"/>
-      <c r="B7" s="73"/>
-      <c r="C7" s="72"/>
-      <c r="D7" s="73"/>
-      <c r="E7" s="72"/>
-      <c r="F7" s="73"/>
-      <c r="G7" s="72"/>
-      <c r="H7" s="73"/>
+      <c r="A7" s="60"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="61"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="1"/>
@@ -3296,86 +3296,86 @@
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="60" t="s">
+      <c r="A9" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="60"/>
-      <c r="C9" s="60"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="60"/>
-      <c r="G9" s="60"/>
-      <c r="H9" s="60"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
     </row>
     <row r="10" spans="1:8" ht="28.05" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="62"/>
-      <c r="G10" s="62"/>
-      <c r="H10" s="63"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="65"/>
     </row>
     <row r="11" spans="1:8" ht="28.05" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="64" t="s">
+      <c r="B11" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65"/>
-      <c r="H11" s="66"/>
+      <c r="C11" s="67"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="67"/>
+      <c r="F11" s="67"/>
+      <c r="G11" s="67"/>
+      <c r="H11" s="68"/>
     </row>
     <row r="12" spans="1:8" ht="28.05" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="64" t="s">
+      <c r="B12" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="66"/>
+      <c r="C12" s="67"/>
+      <c r="D12" s="67"/>
+      <c r="E12" s="67"/>
+      <c r="F12" s="67"/>
+      <c r="G12" s="67"/>
+      <c r="H12" s="68"/>
     </row>
     <row r="13" spans="1:8" ht="28.05" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="64" t="s">
+      <c r="B13" s="66" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="65"/>
-      <c r="D13" s="65"/>
-      <c r="E13" s="65"/>
-      <c r="F13" s="65"/>
-      <c r="G13" s="65"/>
-      <c r="H13" s="66"/>
+      <c r="C13" s="67"/>
+      <c r="D13" s="67"/>
+      <c r="E13" s="67"/>
+      <c r="F13" s="67"/>
+      <c r="G13" s="67"/>
+      <c r="H13" s="68"/>
     </row>
     <row r="14" spans="1:8" ht="28.05" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="57" t="s">
+      <c r="B14" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="58"/>
-      <c r="D14" s="58"/>
-      <c r="E14" s="58"/>
-      <c r="F14" s="58"/>
-      <c r="G14" s="58"/>
-      <c r="H14" s="59"/>
+      <c r="C14" s="72"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="72"/>
+      <c r="F14" s="72"/>
+      <c r="G14" s="72"/>
+      <c r="H14" s="73"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="1"/>
@@ -3388,86 +3388,86 @@
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="60" t="s">
+      <c r="A16" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
-      <c r="H16" s="60"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="62"/>
+      <c r="D16" s="62"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
+      <c r="G16" s="62"/>
+      <c r="H16" s="62"/>
     </row>
     <row r="17" spans="1:8" ht="28.05" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="55"/>
-      <c r="D17" s="55"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="55"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="55"/>
+      <c r="C17" s="69"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="69"/>
+      <c r="F17" s="69"/>
+      <c r="G17" s="69"/>
+      <c r="H17" s="69"/>
     </row>
     <row r="18" spans="1:8" ht="28.05" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="55" t="s">
+      <c r="B18" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="55"/>
-      <c r="D18" s="55"/>
-      <c r="E18" s="55"/>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
+      <c r="C18" s="69"/>
+      <c r="D18" s="69"/>
+      <c r="E18" s="69"/>
+      <c r="F18" s="69"/>
+      <c r="G18" s="69"/>
+      <c r="H18" s="69"/>
     </row>
     <row r="19" spans="1:8" ht="28.05" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="55" t="s">
+      <c r="B19" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="55"/>
-      <c r="D19" s="55"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="55"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="69"/>
+      <c r="G19" s="69"/>
+      <c r="H19" s="69"/>
     </row>
     <row r="20" spans="1:8" ht="28.05" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="55"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
+      <c r="C20" s="69"/>
+      <c r="D20" s="69"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="69"/>
+      <c r="G20" s="69"/>
+      <c r="H20" s="69"/>
     </row>
     <row r="21" spans="1:8" ht="28.05" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="55" t="s">
+      <c r="B21" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="55"/>
-      <c r="D21" s="55"/>
-      <c r="E21" s="55"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="55"/>
+      <c r="C21" s="69"/>
+      <c r="D21" s="69"/>
+      <c r="E21" s="69"/>
+      <c r="F21" s="69"/>
+      <c r="G21" s="69"/>
+      <c r="H21" s="69"/>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="1"/>
@@ -3480,19 +3480,32 @@
       <c r="H22" s="1"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="56" t="s">
+      <c r="A23" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="56"/>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
+      <c r="B23" s="70"/>
+      <c r="C23" s="70"/>
+      <c r="D23" s="70"/>
+      <c r="E23" s="70"/>
+      <c r="F23" s="70"/>
+      <c r="G23" s="70"/>
+      <c r="H23" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B13:H13"/>
     <mergeCell ref="A1:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A5:B5"/>
@@ -3503,19 +3516,6 @@
     <mergeCell ref="E6:F7"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H7"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11331,7 +11331,7 @@
         <v>0.56756756756756754</v>
       </c>
       <c r="L3" s="36">
-        <f t="shared" si="1"/>
+        <f>IF(K3="","",K3*G3)</f>
         <v>0.56756756756756754</v>
       </c>
       <c r="M3" s="25" t="s">
@@ -11457,7 +11457,7 @@
         <v>0.49000000000000005</v>
       </c>
       <c r="K5" s="36">
-        <f t="shared" si="2"/>
+        <f>IF(OR(H5="",F5=""),"",F5*J5/(1-F5*H5))</f>
         <v>0.31779966370405965</v>
       </c>
       <c r="L5" s="36">

</xml_diff>

<commit_message>
no changes but before demographic aligment
</commit_message>
<xml_diff>
--- a/data/indonesia_model_inputs.xlsx
+++ b/data/indonesia_model_inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/WorldBank-Indonesia/uw-wb-indonesia-ncd/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_0C710D44475D1BAD4A588195A28C8E47DB0B7F50" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8523B379-E550-4158-B9D4-5582EA6E3F24}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="11_0C710D44475D1BAD4A588195A28C8E47DB0B7F50" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{750E90AA-655D-4094-A57B-B11ABC5631F6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="FairChoices_Methods" sheetId="9" r:id="rId9"/>
     <sheet name="Scope_and_Sources" sheetId="10" r:id="rId10"/>
     <sheet name="QA_Checks" sheetId="11" r:id="rId11"/>
+    <sheet name="ChangesLog" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,8 +43,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={65F284AB-064D-4B9D-A390-F156B89E3B37}</author>
+  </authors>
+  <commentList>
+    <comment ref="S33" authorId="0" shapeId="0" xr:uid="{65F284AB-064D-4B9D-A390-F156B89E3B37}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Pending update with Sali Info</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1749" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1756" uniqueCount="594">
   <si>
     <t>Indonesia NCD model — user input workbook</t>
   </si>
@@ -1807,6 +1826,24 @@
   </si>
   <si>
     <t>Only selected base-case cost rows are model-ready</t>
+  </si>
+  <si>
+    <t>RHD</t>
+  </si>
+  <si>
+    <t>Cause</t>
+  </si>
+  <si>
+    <t>Intervention</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Since we do not have svere state, the PIN is updated to 9 % based on the RHD detailed model from The Uganda/Indonesia modelling</t>
   </si>
 </sst>
 </file>
@@ -1817,7 +1854,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1881,6 +1918,17 @@
       <i/>
       <sz val="9"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -2115,7 +2163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2279,26 +2327,20 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2321,23 +2363,42 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2751,6 +2812,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="William R Garcia" id="{08755B68-3142-46D3-BD70-CECE36D4D0BB}" userId="S::wrgg@uw.edu::52698913-8803-44d0-b81a-d207944fdb38" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3178,6 +3245,14 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="S33" dT="2026-08-20T17:22:41.38" personId="{08755B68-3142-46D3-BD70-CECE36D4D0BB}" id="{65F284AB-064D-4B9D-A390-F156B89E3B37}">
+    <text>Pending update with Sali Info</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H23"/>
@@ -3192,38 +3267,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="55"/>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
+      <c r="A2" s="67"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="56" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
+      <c r="A3" s="68" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1"/>
@@ -3236,54 +3311,54 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57" t="s">
+      <c r="B5" s="69"/>
+      <c r="C5" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57" t="s">
+      <c r="D5" s="69"/>
+      <c r="E5" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57" t="s">
+      <c r="F5" s="69"/>
+      <c r="G5" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="57"/>
+      <c r="H5" s="69"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="58" t="str">
+      <c r="A6" s="70" t="str">
         <f>IF(COUNTIF(QA_Checks!$E$2:$E$9,"FAIL")=0,"READY TO RUN","REVIEW REQUIRED")</f>
         <v>REVIEW REQUIRED</v>
       </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="58">
+      <c r="B6" s="71"/>
+      <c r="C6" s="70">
         <f>COUNTA(Dictionaries!$A$2:$A$9)</f>
         <v>8</v>
       </c>
-      <c r="D6" s="59"/>
-      <c r="E6" s="58">
+      <c r="D6" s="71"/>
+      <c r="E6" s="70">
         <f>COUNTIF(Dictionaries!$I$2:$I$9,1)</f>
         <v>7</v>
       </c>
-      <c r="F6" s="59"/>
-      <c r="G6" s="58">
+      <c r="F6" s="71"/>
+      <c r="G6" s="70">
         <f>COUNTA(Intervention_Cause_Map!$A$2:$A$18)</f>
         <v>17</v>
       </c>
-      <c r="H6" s="59"/>
+      <c r="H6" s="71"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="60"/>
-      <c r="B7" s="61"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="61"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="61"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="61"/>
+      <c r="A7" s="72"/>
+      <c r="B7" s="73"/>
+      <c r="C7" s="72"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="72"/>
+      <c r="F7" s="73"/>
+      <c r="G7" s="72"/>
+      <c r="H7" s="73"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="1"/>
@@ -3296,86 +3371,86 @@
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="62" t="s">
+      <c r="A9" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="62"/>
-      <c r="C9" s="62"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="62"/>
-      <c r="F9" s="62"/>
-      <c r="G9" s="62"/>
-      <c r="H9" s="62"/>
+      <c r="B9" s="60"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="60"/>
     </row>
     <row r="10" spans="1:8" ht="28.05" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="63" t="s">
+      <c r="B10" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
-      <c r="G10" s="64"/>
-      <c r="H10" s="65"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="63"/>
     </row>
     <row r="11" spans="1:8" ht="28.05" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="66" t="s">
+      <c r="B11" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="67"/>
-      <c r="D11" s="67"/>
-      <c r="E11" s="67"/>
-      <c r="F11" s="67"/>
-      <c r="G11" s="67"/>
-      <c r="H11" s="68"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="66"/>
     </row>
     <row r="12" spans="1:8" ht="28.05" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="66" t="s">
+      <c r="B12" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="67"/>
-      <c r="D12" s="67"/>
-      <c r="E12" s="67"/>
-      <c r="F12" s="67"/>
-      <c r="G12" s="67"/>
-      <c r="H12" s="68"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="65"/>
+      <c r="F12" s="65"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="66"/>
     </row>
     <row r="13" spans="1:8" ht="28.05" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="66" t="s">
+      <c r="B13" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="67"/>
-      <c r="D13" s="67"/>
-      <c r="E13" s="67"/>
-      <c r="F13" s="67"/>
-      <c r="G13" s="67"/>
-      <c r="H13" s="68"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="65"/>
+      <c r="E13" s="65"/>
+      <c r="F13" s="65"/>
+      <c r="G13" s="65"/>
+      <c r="H13" s="66"/>
     </row>
     <row r="14" spans="1:8" ht="28.05" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="71" t="s">
+      <c r="B14" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="72"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="72"/>
-      <c r="F14" s="72"/>
-      <c r="G14" s="72"/>
-      <c r="H14" s="73"/>
+      <c r="C14" s="58"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="59"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="1"/>
@@ -3388,86 +3463,86 @@
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="62" t="s">
+      <c r="A16" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
-      <c r="D16" s="62"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="62"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
+      <c r="B16" s="60"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="60"/>
     </row>
     <row r="17" spans="1:8" ht="28.05" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="69" t="s">
+      <c r="B17" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="69"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="69"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="69"/>
+      <c r="C17" s="55"/>
+      <c r="D17" s="55"/>
+      <c r="E17" s="55"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="55"/>
+      <c r="H17" s="55"/>
     </row>
     <row r="18" spans="1:8" ht="28.05" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="69" t="s">
+      <c r="B18" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="69"/>
-      <c r="D18" s="69"/>
-      <c r="E18" s="69"/>
-      <c r="F18" s="69"/>
-      <c r="G18" s="69"/>
-      <c r="H18" s="69"/>
+      <c r="C18" s="55"/>
+      <c r="D18" s="55"/>
+      <c r="E18" s="55"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="55"/>
+      <c r="H18" s="55"/>
     </row>
     <row r="19" spans="1:8" ht="28.05" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="69" t="s">
+      <c r="B19" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="69"/>
-      <c r="D19" s="69"/>
-      <c r="E19" s="69"/>
-      <c r="F19" s="69"/>
-      <c r="G19" s="69"/>
-      <c r="H19" s="69"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="55"/>
+      <c r="F19" s="55"/>
+      <c r="G19" s="55"/>
+      <c r="H19" s="55"/>
     </row>
     <row r="20" spans="1:8" ht="28.05" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="69" t="s">
+      <c r="B20" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="69"/>
-      <c r="D20" s="69"/>
-      <c r="E20" s="69"/>
-      <c r="F20" s="69"/>
-      <c r="G20" s="69"/>
-      <c r="H20" s="69"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="55"/>
     </row>
     <row r="21" spans="1:8" ht="28.05" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="69" t="s">
+      <c r="B21" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="69"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="69"/>
-      <c r="H21" s="69"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="55"/>
+      <c r="H21" s="55"/>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="1"/>
@@ -3480,32 +3555,19 @@
       <c r="H22" s="1"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="70" t="s">
+      <c r="A23" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="70"/>
-      <c r="C23" s="70"/>
-      <c r="D23" s="70"/>
-      <c r="E23" s="70"/>
-      <c r="F23" s="70"/>
-      <c r="G23" s="70"/>
-      <c r="H23" s="70"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B13:H13"/>
     <mergeCell ref="A1:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A5:B5"/>
@@ -3516,6 +3578,19 @@
     <mergeCell ref="E6:F7"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H7"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3874,11 +3949,11 @@
       </c>
       <c r="D4" s="54">
         <f>COUNTIF(Coverage!$S$2:$S$18,"&lt;&gt;OK")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E4" s="54" t="str">
         <f t="shared" si="0"/>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="F4" s="53" t="s">
         <v>572</v>
@@ -3896,7 +3971,7 @@
       </c>
       <c r="D5" s="54">
         <f>COUNTIF(Cost_Components!$AC$2:$AC$35,"&lt;&gt;OK")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="54" t="str">
         <f t="shared" si="0"/>
@@ -4005,6 +4080,47 @@
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F251E35-2D95-4CA4-949B-9CA41039AC58}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <cols>
+    <col min="2" max="2" width="17.796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>589</v>
+      </c>
+      <c r="B1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C1" t="s">
+        <v>591</v>
+      </c>
+      <c r="D1" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>588</v>
+      </c>
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="75">
+        <v>46254</v>
+      </c>
+      <c r="D2" t="s">
+        <v>593</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -5635,7 +5751,7 @@
         <v>0.75</v>
       </c>
       <c r="K3" s="14">
-        <v>1</v>
+        <v>0.09</v>
       </c>
       <c r="L3" s="33">
         <v>5</v>
@@ -7787,7 +7903,9 @@
       <c r="F17" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="G17" s="14"/>
+      <c r="G17" s="76">
+        <v>0.31</v>
+      </c>
       <c r="H17" s="14"/>
       <c r="I17" s="36">
         <f>IF(H17="",Assumptions!$B$5,H17)</f>
@@ -7812,9 +7930,9 @@
       <c r="P17" s="9" t="s">
         <v>286</v>
       </c>
-      <c r="Q17" s="36" t="str">
+      <c r="Q17" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.49000000000000005</v>
       </c>
       <c r="R17" s="25">
         <f>COUNTIF(Intervention_Cause_Map!$A$2:$A$18,B17)</f>
@@ -7822,7 +7940,7 @@
       </c>
       <c r="S17" s="25" t="str">
         <f t="shared" si="1"/>
-        <v>MISSING BASELINE</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="22.8">
@@ -7844,7 +7962,9 @@
       <c r="F18" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="G18" s="31"/>
+      <c r="G18" s="76">
+        <v>0.31</v>
+      </c>
       <c r="H18" s="31"/>
       <c r="I18" s="37">
         <f>IF(H18="",Assumptions!$B$5,H18)</f>
@@ -7869,9 +7989,9 @@
       <c r="P18" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="Q18" s="37" t="str">
+      <c r="Q18" s="37">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.49000000000000005</v>
       </c>
       <c r="R18" s="26">
         <f>COUNTIF(Intervention_Cause_Map!$A$2:$A$18,B18)</f>
@@ -7879,7 +7999,7 @@
       </c>
       <c r="S18" s="26" t="str">
         <f t="shared" si="1"/>
-        <v>MISSING BASELINE</v>
+        <v>OK</v>
       </c>
     </row>
   </sheetData>
@@ -7903,7 +8023,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AC35"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
@@ -10862,8 +10982,8 @@
       <c r="C33" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D33" s="33">
-        <v>0</v>
+      <c r="D33" s="78">
+        <v>1</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>118</v>
@@ -10907,7 +11027,9 @@
       <c r="R33" s="9" t="s">
         <v>317</v>
       </c>
-      <c r="S33" s="42"/>
+      <c r="S33" s="77">
+        <v>7</v>
+      </c>
       <c r="T33" s="12">
         <v>2023</v>
       </c>
@@ -10933,11 +11055,11 @@
       </c>
       <c r="AB33" s="25">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC33" s="25" t="str">
-        <f t="shared" si="1"/>
-        <v>MISSING COST</v>
+        <f>IF(AA33&lt;1,"BAD KEY",IF(S33="","MISSING COST",IF(U33=0,"REVIEW ADJUSTMENT",IF(AB33&lt;&gt;1,"CHECK SELECTION","OK"))))</f>
+        <v>OK</v>
       </c>
     </row>
     <row r="34" spans="1:29">
@@ -11040,7 +11162,7 @@
       <c r="C35" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="D35" s="34">
+      <c r="D35" s="79">
         <v>1</v>
       </c>
       <c r="E35" s="10" t="s">
@@ -11118,7 +11240,7 @@
         <v>1</v>
       </c>
       <c r="AC35" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(AA35&lt;1,"BAD KEY",IF(S35="","MISSING COST",IF(U35=0,"REVIEW ADJUSTMENT",IF(AB35&lt;&gt;1,"CHECK SELECTION","OK"))))</f>
         <v>REVIEW ADJUSTMENT</v>
       </c>
     </row>
@@ -11141,8 +11263,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11312,7 +11435,7 @@
       </c>
       <c r="G3" s="36">
         <f>SUMIF(Effect_Sizes!$B$2:$B$18,A3,Effect_Sizes!$K$2:$K$18)</f>
-        <v>1</v>
+        <v>0.09</v>
       </c>
       <c r="H3" s="36">
         <f>SUMIF(Coverage!$B$2:$B$18,A3,Coverage!$G$2:$G$18)</f>
@@ -11332,7 +11455,7 @@
       </c>
       <c r="L3" s="36">
         <f>IF(K3="","",K3*G3)</f>
-        <v>0.56756756756756754</v>
+        <v>5.108108108108108E-2</v>
       </c>
       <c r="M3" s="25" t="s">
         <v>142</v>
@@ -12057,11 +12180,11 @@
       </c>
       <c r="O14" s="39">
         <f>COUNTIFS(Cost_Components!$G$2:$G$35,M14,Cost_Components!$D$2:$D$35,1)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="45">
         <f>SUMIFS(Cost_Components!$S$2:$S$35,Cost_Components!$G$2:$G$35,M14,Cost_Components!$D$2:$D$35,1)</f>
-        <v>34.349530000000001</v>
+        <v>41.349530000000001</v>
       </c>
       <c r="Q14" s="25" t="str">
         <f>IF(H14=0,"MISSING COVERAGE",IF(O14=0,"REVIEW COST",IF(COUNTIF(Effect_Sizes!$B$2:$B$18,A14)&lt;&gt;1,"BAD EFFECT KEY","REVIEWED LINK")))</f>
@@ -12226,7 +12349,7 @@
       </c>
       <c r="H17" s="36">
         <f>SUMIF(Coverage!$B$2:$B$18,A17,Coverage!$G$2:$G$18)</f>
-        <v>0</v>
+        <v>0.31</v>
       </c>
       <c r="I17" s="36">
         <f>SUMIF(Coverage!$B$2:$B$18,A17,Coverage!$I$2:$I$18)</f>
@@ -12234,15 +12357,15 @@
       </c>
       <c r="J17" s="36">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.49000000000000005</v>
       </c>
       <c r="K17" s="36">
         <f t="shared" si="2"/>
-        <v>0.22400000000000003</v>
+        <v>0.15024091108190979</v>
       </c>
       <c r="L17" s="36">
         <f t="shared" si="1"/>
-        <v>0.22400000000000003</v>
+        <v>0.15024091108190979</v>
       </c>
       <c r="M17" s="25" t="s">
         <v>165</v>
@@ -12260,7 +12383,7 @@
       </c>
       <c r="Q17" s="25" t="str">
         <f>IF(H17=0,"MISSING COVERAGE",IF(O17=0,"REVIEW COST",IF(COUNTIF(Effect_Sizes!$B$2:$B$18,A17)&lt;&gt;1,"BAD EFFECT KEY","REVIEWED LINK")))</f>
-        <v>MISSING COVERAGE</v>
+        <v>REVIEWED LINK</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="22.8">
@@ -12291,7 +12414,7 @@
       </c>
       <c r="H18" s="37">
         <f>SUMIF(Coverage!$B$2:$B$18,A18,Coverage!$G$2:$G$18)</f>
-        <v>0</v>
+        <v>0.31</v>
       </c>
       <c r="I18" s="37">
         <f>SUMIF(Coverage!$B$2:$B$18,A18,Coverage!$I$2:$I$18)</f>
@@ -12299,15 +12422,15 @@
       </c>
       <c r="J18" s="37">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.49000000000000005</v>
       </c>
       <c r="K18" s="37">
         <f t="shared" si="2"/>
-        <v>0.12</v>
+        <v>7.7084425799685385E-2</v>
       </c>
       <c r="L18" s="37">
         <f t="shared" si="1"/>
-        <v>1.7999999999999999E-2</v>
+        <v>1.1562663869952807E-2</v>
       </c>
       <c r="M18" s="26" t="s">
         <v>165</v>
@@ -12325,7 +12448,7 @@
       </c>
       <c r="Q18" s="26" t="str">
         <f>IF(H18=0,"MISSING COVERAGE",IF(O18=0,"REVIEW COST",IF(COUNTIF(Effect_Sizes!$B$2:$B$18,A18)&lt;&gt;1,"BAD EFFECT KEY","REVIEWED LINK")))</f>
-        <v>MISSING COVERAGE</v>
+        <v>REVIEWED LINK</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lock presentation code and zili's frp inputs
</commit_message>
<xml_diff>
--- a/data/indonesia_model_inputs.xlsx
+++ b/data/indonesia_model_inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/WorldBank-Indonesia/uw-wb-indonesia-ncd/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_DC2E0DB659B3F61906DA456628709D9ECC8254F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E7A28FC-523C-415C-8B2E-3C381431A492}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_DC2E0DB659B3F61906DA456628709D9ECC8254F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8414A789-FA28-4929-A274-73F215098615}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -7684,7 +7684,7 @@
       <c r="G3" s="26">
         <v>0.1</v>
       </c>
-      <c r="H3" s="26"/>
+      <c r="H3" s="27"/>
       <c r="I3" s="33">
         <f>IF(H3="",Assumptions!$B$5,H3)</f>
         <v>0.8</v>
@@ -7747,7 +7747,7 @@
       <c r="G4" s="26">
         <v>0.31</v>
       </c>
-      <c r="H4" s="26"/>
+      <c r="H4" s="27"/>
       <c r="I4" s="33">
         <f>IF(H4="",Assumptions!$B$5,H4)</f>
         <v>0.8</v>
@@ -7810,7 +7810,7 @@
       <c r="G5" s="26">
         <v>0.31</v>
       </c>
-      <c r="H5" s="26"/>
+      <c r="H5" s="27"/>
       <c r="I5" s="33">
         <f>IF(H5="",Assumptions!$B$5,H5)</f>
         <v>0.8</v>
@@ -7873,7 +7873,7 @@
       <c r="G6" s="26">
         <v>0.31</v>
       </c>
-      <c r="H6" s="26"/>
+      <c r="H6" s="27"/>
       <c r="I6" s="33">
         <f>IF(H6="",Assumptions!$B$5,H6)</f>
         <v>0.8</v>
@@ -7936,7 +7936,7 @@
       <c r="G7" s="26">
         <v>0.31</v>
       </c>
-      <c r="H7" s="26"/>
+      <c r="H7" s="27"/>
       <c r="I7" s="33">
         <f>IF(H7="",Assumptions!$B$5,H7)</f>
         <v>0.8</v>
@@ -7999,7 +7999,7 @@
       <c r="G8" s="26">
         <v>0.31</v>
       </c>
-      <c r="H8" s="26"/>
+      <c r="H8" s="27"/>
       <c r="I8" s="33">
         <f>IF(H8="",Assumptions!$B$5,H8)</f>
         <v>0.8</v>
@@ -8062,7 +8062,7 @@
       <c r="G9" s="26">
         <v>0.31</v>
       </c>
-      <c r="H9" s="26"/>
+      <c r="H9" s="27"/>
       <c r="I9" s="33">
         <f>IF(H9="",Assumptions!$B$5,H9)</f>
         <v>0.8</v>
@@ -8125,7 +8125,7 @@
       <c r="G10" s="26">
         <v>0.31</v>
       </c>
-      <c r="H10" s="26"/>
+      <c r="H10" s="27"/>
       <c r="I10" s="33">
         <f>IF(H10="",Assumptions!$B$5,H10)</f>
         <v>0.8</v>
@@ -8188,7 +8188,7 @@
       <c r="G11" s="26">
         <v>0.31</v>
       </c>
-      <c r="H11" s="26"/>
+      <c r="H11" s="27"/>
       <c r="I11" s="33">
         <f>IF(H11="",Assumptions!$B$5,H11)</f>
         <v>0.8</v>
@@ -8251,7 +8251,7 @@
       <c r="G12" s="26">
         <v>0.31</v>
       </c>
-      <c r="H12" s="26"/>
+      <c r="H12" s="27"/>
       <c r="I12" s="33">
         <f>IF(H12="",Assumptions!$B$5,H12)</f>
         <v>0.8</v>
@@ -8314,7 +8314,7 @@
       <c r="G13" s="26">
         <v>0.31</v>
       </c>
-      <c r="H13" s="26"/>
+      <c r="H13" s="27"/>
       <c r="I13" s="33">
         <f>IF(H13="",Assumptions!$B$5,H13)</f>
         <v>0.8</v>
@@ -8377,7 +8377,7 @@
       <c r="G14" s="26">
         <v>0.31</v>
       </c>
-      <c r="H14" s="26"/>
+      <c r="H14" s="27"/>
       <c r="I14" s="33">
         <f>IF(H14="",Assumptions!$B$5,H14)</f>
         <v>0.8</v>
@@ -8440,7 +8440,7 @@
       <c r="G15" s="26">
         <v>0.31</v>
       </c>
-      <c r="H15" s="26"/>
+      <c r="H15" s="27"/>
       <c r="I15" s="33">
         <f>IF(H15="",Assumptions!$B$5,H15)</f>
         <v>0.8</v>
@@ -8503,7 +8503,7 @@
       <c r="G16" s="26">
         <v>0.31</v>
       </c>
-      <c r="H16" s="26"/>
+      <c r="H16" s="27"/>
       <c r="I16" s="33">
         <f>IF(H16="",Assumptions!$B$5,H16)</f>
         <v>0.8</v>
@@ -8566,7 +8566,7 @@
       <c r="G17" s="38">
         <v>0.31</v>
       </c>
-      <c r="H17" s="26"/>
+      <c r="H17" s="27"/>
       <c r="I17" s="33">
         <f>IF(H17="",Assumptions!$B$5,H17)</f>
         <v>0.8</v>
@@ -8625,7 +8625,7 @@
       <c r="G18" s="38">
         <v>0.31</v>
       </c>
-      <c r="H18" s="28"/>
+      <c r="H18" s="27"/>
       <c r="I18" s="34">
         <f>IF(H18="",Assumptions!$B$5,H18)</f>
         <v>0.8</v>

</xml_diff>

<commit_message>
Include Will's calibrated probabilities and before subnational cascade
</commit_message>
<xml_diff>
--- a/data/indonesia_model_inputs.xlsx
+++ b/data/indonesia_model_inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/WorldBank-Indonesia/uw-wb-indonesia-ncd/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_45329FAA1C5950AFA18B860B8102B22A93A6ACC6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5DCF537-D55D-4731-AC69-4177EBDC4BD9}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="11_45329FAA1C5950AFA18B860B8102B22A93A6ACC6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCC6E55B-2FE9-4B6D-A1A9-54BE5C9A9A4C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -67,13 +67,22 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={B1FEFC56-CF80-485C-B87E-A5E63818491E}</author>
     <author>tc={5282C296-63F9-415C-B2F2-3B273B7413D7}</author>
     <author>tc={D51D381D-3B39-435F-B5B2-6143D8D91563}</author>
     <author>tc={65F284AB-064D-4B9D-A390-F156B89E3B37}</author>
     <author>tc={8DE0ED5B-C37D-4E7B-B75F-DADA3DBFFB3B}</author>
   </authors>
   <commentList>
-    <comment ref="L6" authorId="0" shapeId="0" xr:uid="{5282C296-63F9-415C-B2F2-3B273B7413D7}">
+    <comment ref="L3" authorId="0" shapeId="0" xr:uid="{B1FEFC56-CF80-485C-B87E-A5E63818491E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    PIN 10%, but *.41 because those are the severe cases</t>
+      </text>
+    </comment>
+    <comment ref="L6" authorId="1" shapeId="0" xr:uid="{5282C296-63F9-415C-B2F2-3B273B7413D7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -81,7 +90,7 @@
     Raised from 6% to 30%</t>
       </text>
     </comment>
-    <comment ref="O8" authorId="1" shapeId="0" xr:uid="{D51D381D-3B39-435F-B5B2-6143D8D91563}">
+    <comment ref="O8" authorId="2" shapeId="0" xr:uid="{D51D381D-3B39-435F-B5B2-6143D8D91563}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -89,7 +98,7 @@
     Updated from 0</t>
       </text>
     </comment>
-    <comment ref="S33" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0600-000001000000}">
+    <comment ref="S33" authorId="3" shapeId="0" xr:uid="{00000000-0006-0000-0600-000001000000}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -97,7 +106,7 @@
     Pending update with Sali Info</t>
       </text>
     </comment>
-    <comment ref="L35" authorId="3" shapeId="0" xr:uid="{8DE0ED5B-C37D-4E7B-B75F-DADA3DBFFB3B}">
+    <comment ref="L35" authorId="4" shapeId="0" xr:uid="{8DE0ED5B-C37D-4E7B-B75F-DADA3DBFFB3B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -2199,7 +2208,7 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2617,20 +2626,33 @@
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2653,36 +2675,23 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3341,6 +3350,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA9DEF6B-1F41-0FC3-6761-D6F769C9562E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7620000" cy="7620000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3786,6 +3849,9 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="L3" dT="2026-08-28T21:04:09.70" personId="{AE4CD8BF-B03D-4C3B-B05E-44787D7972AD}" id="{B1FEFC56-CF80-485C-B87E-A5E63818491E}">
+    <text>PIN 10%, but *.41 because those are the severe cases</text>
+  </threadedComment>
   <threadedComment ref="L6" dT="2026-08-28T18:06:24.02" personId="{AE4CD8BF-B03D-4C3B-B05E-44787D7972AD}" id="{5282C296-63F9-415C-B2F2-3B273B7413D7}">
     <text>Raised from 6% to 30%</text>
   </threadedComment>
@@ -3818,38 +3884,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="73"/>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
+      <c r="A2" s="64"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="74" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
-      <c r="G3" s="74"/>
-      <c r="H3" s="74"/>
+      <c r="A3" s="65" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1"/>
@@ -3862,54 +3928,54 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75" t="s">
+      <c r="B5" s="66"/>
+      <c r="C5" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75" t="s">
+      <c r="D5" s="66"/>
+      <c r="E5" s="66" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75" t="s">
+      <c r="F5" s="66"/>
+      <c r="G5" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="75"/>
+      <c r="H5" s="66"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="76" t="str">
+      <c r="A6" s="67" t="str">
         <f>IF(COUNTIF(QA_Checks!$E$2:$E$9,"FAIL")=0,"READY TO RUN","REVIEW REQUIRED")</f>
         <v>READY TO RUN</v>
       </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="76">
+      <c r="B6" s="68"/>
+      <c r="C6" s="67">
         <f>COUNTA(Dictionaries!$A$2:$A$9)</f>
         <v>8</v>
       </c>
-      <c r="D6" s="77"/>
-      <c r="E6" s="76">
+      <c r="D6" s="68"/>
+      <c r="E6" s="67">
         <f>COUNTIF(Dictionaries!$I$2:$I$9,1)</f>
         <v>7</v>
       </c>
-      <c r="F6" s="77"/>
-      <c r="G6" s="76">
+      <c r="F6" s="68"/>
+      <c r="G6" s="67">
         <f>COUNTA(Intervention_Cause_Map!$A$2:$A$18)</f>
         <v>17</v>
       </c>
-      <c r="H6" s="77"/>
+      <c r="H6" s="68"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="78"/>
-      <c r="B7" s="79"/>
-      <c r="C7" s="78"/>
-      <c r="D7" s="79"/>
-      <c r="E7" s="78"/>
-      <c r="F7" s="79"/>
-      <c r="G7" s="78"/>
-      <c r="H7" s="79"/>
+      <c r="A7" s="69"/>
+      <c r="B7" s="70"/>
+      <c r="C7" s="69"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="69"/>
+      <c r="H7" s="70"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="1"/>
@@ -3922,86 +3988,86 @@
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="66" t="s">
+      <c r="A9" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="66"/>
-      <c r="C9" s="66"/>
-      <c r="D9" s="66"/>
-      <c r="E9" s="66"/>
-      <c r="F9" s="66"/>
-      <c r="G9" s="66"/>
-      <c r="H9" s="66"/>
+      <c r="B9" s="71"/>
+      <c r="C9" s="71"/>
+      <c r="D9" s="71"/>
+      <c r="E9" s="71"/>
+      <c r="F9" s="71"/>
+      <c r="G9" s="71"/>
+      <c r="H9" s="71"/>
     </row>
     <row r="10" spans="1:8" ht="28.05" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="67" t="s">
+      <c r="B10" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="68"/>
-      <c r="F10" s="68"/>
-      <c r="G10" s="68"/>
-      <c r="H10" s="69"/>
+      <c r="C10" s="73"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="73"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:8" ht="28.05" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="70" t="s">
+      <c r="B11" s="75" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="71"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="71"/>
-      <c r="F11" s="71"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="72"/>
+      <c r="C11" s="76"/>
+      <c r="D11" s="76"/>
+      <c r="E11" s="76"/>
+      <c r="F11" s="76"/>
+      <c r="G11" s="76"/>
+      <c r="H11" s="77"/>
     </row>
     <row r="12" spans="1:8" ht="28.05" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="70" t="s">
+      <c r="B12" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="71"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="71"/>
-      <c r="F12" s="71"/>
-      <c r="G12" s="71"/>
-      <c r="H12" s="72"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
+      <c r="F12" s="76"/>
+      <c r="G12" s="76"/>
+      <c r="H12" s="77"/>
     </row>
     <row r="13" spans="1:8" ht="28.05" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="70" t="s">
+      <c r="B13" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="71"/>
-      <c r="D13" s="71"/>
-      <c r="E13" s="71"/>
-      <c r="F13" s="71"/>
-      <c r="G13" s="71"/>
-      <c r="H13" s="72"/>
+      <c r="C13" s="76"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="76"/>
+      <c r="F13" s="76"/>
+      <c r="G13" s="76"/>
+      <c r="H13" s="77"/>
     </row>
     <row r="14" spans="1:8" ht="28.05" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="63" t="s">
+      <c r="B14" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="64"/>
-      <c r="G14" s="64"/>
-      <c r="H14" s="65"/>
+      <c r="C14" s="81"/>
+      <c r="D14" s="81"/>
+      <c r="E14" s="81"/>
+      <c r="F14" s="81"/>
+      <c r="G14" s="81"/>
+      <c r="H14" s="82"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="1"/>
@@ -4014,86 +4080,86 @@
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="66" t="s">
+      <c r="A16" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="66"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
-      <c r="G16" s="66"/>
-      <c r="H16" s="66"/>
+      <c r="B16" s="71"/>
+      <c r="C16" s="71"/>
+      <c r="D16" s="71"/>
+      <c r="E16" s="71"/>
+      <c r="F16" s="71"/>
+      <c r="G16" s="71"/>
+      <c r="H16" s="71"/>
     </row>
     <row r="17" spans="1:8" ht="28.05" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>622</v>
       </c>
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="78" t="s">
         <v>623</v>
       </c>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
+      <c r="C17" s="78"/>
+      <c r="D17" s="78"/>
+      <c r="E17" s="78"/>
+      <c r="F17" s="78"/>
+      <c r="G17" s="78"/>
+      <c r="H17" s="78"/>
     </row>
     <row r="18" spans="1:8" ht="28.05" customHeight="1">
       <c r="A18" s="3" t="s">
         <v>622</v>
       </c>
-      <c r="B18" s="61" t="s">
+      <c r="B18" s="78" t="s">
         <v>624</v>
       </c>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
+      <c r="C18" s="78"/>
+      <c r="D18" s="78"/>
+      <c r="E18" s="78"/>
+      <c r="F18" s="78"/>
+      <c r="G18" s="78"/>
+      <c r="H18" s="78"/>
     </row>
     <row r="19" spans="1:8" ht="28.05" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="61"/>
-      <c r="D19" s="61"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="61"/>
-      <c r="G19" s="61"/>
-      <c r="H19" s="61"/>
+      <c r="C19" s="78"/>
+      <c r="D19" s="78"/>
+      <c r="E19" s="78"/>
+      <c r="F19" s="78"/>
+      <c r="G19" s="78"/>
+      <c r="H19" s="78"/>
     </row>
     <row r="20" spans="1:8" ht="28.05" customHeight="1">
       <c r="A20" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="78" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="61"/>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="61"/>
-      <c r="H20" s="61"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="78"/>
+      <c r="E20" s="78"/>
+      <c r="F20" s="78"/>
+      <c r="G20" s="78"/>
+      <c r="H20" s="78"/>
     </row>
     <row r="21" spans="1:8" ht="28.05" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="78" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="61"/>
-      <c r="D21" s="61"/>
-      <c r="E21" s="61"/>
-      <c r="F21" s="61"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="61"/>
+      <c r="C21" s="78"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="78"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="78"/>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="1"/>
@@ -4106,19 +4172,32 @@
       <c r="H22" s="1"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="62" t="s">
+      <c r="A23" s="79" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="62"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="62"/>
+      <c r="B23" s="79"/>
+      <c r="C23" s="79"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="79"/>
+      <c r="F23" s="79"/>
+      <c r="G23" s="79"/>
+      <c r="H23" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B13:H13"/>
     <mergeCell ref="A1:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A5:B5"/>
@@ -4129,19 +4208,6 @@
     <mergeCell ref="E6:F7"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H7"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B19:H19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4691,7 +4757,7 @@
       <c r="B4" t="s">
         <v>660</v>
       </c>
-      <c r="C4" s="81">
+      <c r="C4" s="61">
         <v>46262</v>
       </c>
       <c r="D4" t="s">
@@ -4705,7 +4771,7 @@
       <c r="B5" t="s">
         <v>663</v>
       </c>
-      <c r="C5" s="81">
+      <c r="C5" s="61">
         <v>46263</v>
       </c>
       <c r="D5" t="s">
@@ -9297,7 +9363,8 @@
         <v>350</v>
       </c>
       <c r="L3" s="26">
-        <v>0.1</v>
+        <f>10%*0.41</f>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="M3" s="18" t="s">
         <v>359</v>
@@ -9766,7 +9833,7 @@
       <c r="N8" s="30">
         <v>1</v>
       </c>
-      <c r="O8" s="82">
+      <c r="O8" s="62">
         <v>30</v>
       </c>
       <c r="P8" s="24">
@@ -9858,7 +9925,7 @@
       <c r="N9" s="30">
         <v>1</v>
       </c>
-      <c r="O9" s="82">
+      <c r="O9" s="62">
         <v>30</v>
       </c>
       <c r="P9" s="24">
@@ -9950,7 +10017,7 @@
       <c r="N10" s="30">
         <v>1</v>
       </c>
-      <c r="O10" s="82">
+      <c r="O10" s="62">
         <v>30</v>
       </c>
       <c r="P10" s="24">
@@ -10042,7 +10109,7 @@
       <c r="N11" s="30">
         <v>1</v>
       </c>
-      <c r="O11" s="82">
+      <c r="O11" s="62">
         <v>30</v>
       </c>
       <c r="P11" s="24">
@@ -12215,7 +12282,7 @@
       <c r="K35" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="L35" s="83">
+      <c r="L35" s="63">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="M35" s="5" t="s">
@@ -13966,14 +14033,14 @@
       <c r="F15" s="53"/>
     </row>
     <row r="17" spans="1:6" ht="34.049999999999997" customHeight="1">
-      <c r="A17" s="80" t="s">
+      <c r="A17" s="83" t="s">
         <v>546</v>
       </c>
-      <c r="B17" s="80"/>
-      <c r="C17" s="80"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="83"/>
+      <c r="E17" s="83"/>
+      <c r="F17" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>